<commit_message>
chinh sua test case
</commit_message>
<xml_diff>
--- a/DOCX/testcasexlsx.xlsx
+++ b/DOCX/testcasexlsx.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="164">
   <si>
     <t>TEST CASE – MULTI-FILE UPLOAD CLIENT/SERVER</t>
   </si>
@@ -374,151 +374,142 @@
     <t>CL_15</t>
   </si>
   <si>
-    <t>Kéo thả file</t>
-  </si>
-  <si>
-    <t>Kéo file vào vùng Drag &amp; Drop Files</t>
+    <t>Clear List</t>
+  </si>
+  <si>
+    <t>Đã có file trong danh sách</t>
+  </si>
+  <si>
+    <t>Nhấn Clear List</t>
   </si>
   <si>
     <t>CL_16</t>
   </si>
   <si>
-    <t>Clear List</t>
-  </si>
-  <si>
-    <t>Đã có file trong danh sách</t>
-  </si>
-  <si>
-    <t>Nhấn Clear List</t>
+    <t>Upload khi chưa kết nối</t>
+  </si>
+  <si>
+    <t>Có file trong danh sách, Client chưa Connected</t>
+  </si>
+  <si>
+    <t>Nhấn Upload</t>
   </si>
   <si>
     <t>CL_17</t>
   </si>
   <si>
-    <t>Upload khi chưa kết nối</t>
-  </si>
-  <si>
-    <t>Có file trong danh sách, Client chưa Connected</t>
-  </si>
-  <si>
-    <t>Nhấn Upload</t>
+    <t>Upload khi chưa chọn file</t>
+  </si>
+  <si>
+    <t>Client đã Connected, danh sách file trống</t>
   </si>
   <si>
     <t>CL_18</t>
   </si>
   <si>
-    <t>Upload khi chưa chọn file</t>
-  </si>
-  <si>
-    <t>Client đã Connected, danh sách file trống</t>
+    <t>Upload 1 file thành công</t>
+  </si>
+  <si>
+    <t>Client Connected, có 1 file</t>
   </si>
   <si>
     <t>CL_19</t>
   </si>
   <si>
-    <t>Upload 1 file thành công</t>
-  </si>
-  <si>
-    <t>Client Connected, có 1 file</t>
+    <t>Upload nhiều file thành công</t>
+  </si>
+  <si>
+    <t>Client Connected, có nhiều file</t>
   </si>
   <si>
     <t>CL_20</t>
   </si>
   <si>
-    <t>Upload nhiều file thành công</t>
-  </si>
-  <si>
-    <t>Client Connected, có nhiều file</t>
+    <t>Hiển thị tiến trình upload</t>
+  </si>
+  <si>
+    <t>Đang upload file</t>
+  </si>
+  <si>
+    <t>Quan sát cột Tiến trình</t>
   </si>
   <si>
     <t>CL_21</t>
   </si>
   <si>
-    <t>Hiển thị tiến trình upload</t>
-  </si>
-  <si>
-    <t>Đang upload file</t>
-  </si>
-  <si>
-    <t>Quan sát cột Tiến trình</t>
+    <t>Pause upload</t>
+  </si>
+  <si>
+    <t>Nhấn Pause</t>
   </si>
   <si>
     <t>CL_22</t>
   </si>
   <si>
-    <t>Pause upload</t>
-  </si>
-  <si>
-    <t>Nhấn Pause</t>
+    <t>Resume upload</t>
+  </si>
+  <si>
+    <t>File đang Paused</t>
+  </si>
+  <si>
+    <t>Nhấn Resume</t>
   </si>
   <si>
     <t>CL_23</t>
   </si>
   <si>
-    <t>Resume upload</t>
-  </si>
-  <si>
-    <t>File đang Paused</t>
-  </si>
-  <si>
-    <t>Nhấn Resume</t>
+    <t>Disconnect khi đang upload</t>
   </si>
   <si>
     <t>CL_24</t>
   </si>
   <si>
-    <t>Disconnect khi đang upload</t>
+    <t>Upload file trùng tên</t>
+  </si>
+  <si>
+    <t>Server đã có file cùng tên</t>
+  </si>
+  <si>
+    <t>Upload lại file cùng tên</t>
   </si>
   <si>
     <t>CL_25</t>
   </si>
   <si>
-    <t>Upload file trùng tên</t>
-  </si>
-  <si>
-    <t>Server đã có file cùng tên</t>
-  </si>
-  <si>
-    <t>Upload lại file cùng tên</t>
+    <t>Upload file dung lượng 0 KB</t>
+  </si>
+  <si>
+    <t>Chọn file rỗng</t>
   </si>
   <si>
     <t>CL_26</t>
   </si>
   <si>
-    <t>Upload file dung lượng 0 KB</t>
-  </si>
-  <si>
-    <t>Chọn file rỗng</t>
+    <t>Upload file lớn</t>
+  </si>
+  <si>
+    <t>Chọn file dung lượng lớn</t>
   </si>
   <si>
     <t>CL_27</t>
   </si>
   <si>
-    <t>Upload file lớn</t>
-  </si>
-  <si>
-    <t>Chọn file dung lượng lớn</t>
+    <t>Upload file có tên tiếng Việt</t>
+  </si>
+  <si>
+    <t>Chọn file tên báo cáo.docx</t>
   </si>
   <si>
     <t>CL_28</t>
   </si>
   <si>
-    <t>Upload file có tên tiếng Việt</t>
-  </si>
-  <si>
-    <t>Chọn file tên báo cáo.docx</t>
+    <t>Upload file có ký tự đặc biệt</t>
+  </si>
+  <si>
+    <t>Chọn file tên test @#$%.txt</t>
   </si>
   <si>
     <t>CL_29</t>
-  </si>
-  <si>
-    <t>Upload file có ký tự đặc biệt</t>
-  </si>
-  <si>
-    <t>Chọn file tên test @#$%.txt</t>
-  </si>
-  <si>
-    <t>CL_30</t>
   </si>
   <si>
     <t>Đóng Client khi đang kết nối</t>
@@ -2233,44 +2224,44 @@
         <v>115</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E35" s="4"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" ht="28.8" spans="1:5">
       <c r="A36" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" ht="28.8" spans="1:5">
       <c r="A37" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="E37" s="4"/>
     </row>
-    <row r="38" ht="28.8" spans="1:5">
+    <row r="38" spans="1:5">
       <c r="A38" s="3" t="s">
         <v>125</v>
       </c>
@@ -2281,7 +2272,7 @@
         <v>127</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E38" s="4"/>
     </row>
@@ -2296,7 +2287,7 @@
         <v>130</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E39" s="4"/>
     </row>
@@ -2311,19 +2302,19 @@
         <v>133</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>137</v>
@@ -2338,55 +2329,55 @@
         <v>139</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="C44" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="D44" s="5" t="s">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="E44" s="4"/>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="E45" s="4"/>
     </row>
@@ -2401,7 +2392,7 @@
         <v>153</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E46" s="4"/>
     </row>
@@ -2416,7 +2407,7 @@
         <v>156</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E47" s="4"/>
     </row>
@@ -2430,8 +2421,8 @@
       <c r="C48" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>124</v>
+      <c r="D48" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="E48" s="4"/>
     </row>
@@ -2446,23 +2437,12 @@
         <v>162</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>124</v>
+        <v>163</v>
       </c>
       <c r="E49" s="4"/>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>166</v>
-      </c>
+      <c r="A50" s="3"/>
       <c r="E50" s="4"/>
     </row>
     <row r="51" spans="1:5">

</xml_diff>